<commit_message>
Final code for manuscript submission to Epilepsia Open
</commit_message>
<xml_diff>
--- a/SDI_comparison_table_Manuscript.xlsx
+++ b/SDI_comparison_table_Manuscript.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -498,9 +498,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="n">
-        <v>-1.14</v>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>-1.01</v>
@@ -555,7 +553,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>-0.71</v>
+        <v>-0.66</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
@@ -610,9 +608,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="n">
-        <v>-0.79</v>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>-0.91</v>
       </c>
@@ -703,7 +699,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>-2.28</v>
+        <v>-2.31</v>
       </c>
       <c r="G16" t="n">
         <v>-2.34</v>
@@ -723,7 +719,7 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
-        <v>-0.68</v>
+        <v>-0.59</v>
       </c>
       <c r="G17" t="n">
         <v>-0.93</v>
@@ -776,7 +772,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-2.36</v>
+        <v>-2.4</v>
       </c>
       <c r="D20" t="n">
         <v>-2.12</v>
@@ -814,7 +810,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-1.91</v>
+        <v>-1.59</v>
       </c>
       <c r="D22" t="n">
         <v>-1.59</v>
@@ -822,9 +818,7 @@
       <c r="E22" t="n">
         <v>-1.57</v>
       </c>
-      <c r="F22" t="n">
-        <v>-0.89</v>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
         <v>-0.88</v>
       </c>
@@ -872,18 +866,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Left-Amygdala</t>
+          <t>transversetemporal_1</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-2.15</v>
-      </c>
-      <c r="D25" t="n">
-        <v>-2.11</v>
-      </c>
-      <c r="E25" t="n">
-        <v>-1.65</v>
-      </c>
+        <v>-0.92</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -894,19 +884,37 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>Left-Amygdala</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>-2.11</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-1.65</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>Left-Hippocampus</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="n">
-        <v>-0.12</v>
-      </c>
-      <c r="G26" t="n">
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
         <v>-0.2</v>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>